<commit_message>
Enhance: Dual-unit gas sales formatting and comprehensive Wellhead Price telemetry
</commit_message>
<xml_diff>
--- a/createpetroleum_2569_8.xlsx
+++ b/createpetroleum_2569_8.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ptitorg.sharepoint.com/sites/PTITFocusStatistics/Shared Documents/General/2026 PTIT Focus/PL/SOURCE/DMF/Production/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_C4A7A707939C26C5AFE036FE6AA9A8AB8208BC02" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF9AEDB7-6F90-4D47-BDFF-714419A460A5}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="23280" windowHeight="12480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="การผลิตปิโตรเลียม" sheetId="1" r:id="rId4"/>
+    <sheet name="การผลิตปิโตรเลียม" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="123">
   <si>
     <t>รายงานปริมาณการผลิตปิโตรเลียม</t>
   </si>
@@ -292,18 +297,6 @@
     <t>2,469.33</t>
   </si>
   <si>
-    <t>430,651.03</t>
-  </si>
-  <si>
-    <t>73,584.55</t>
-  </si>
-  <si>
-    <t>66,932.51</t>
-  </si>
-  <si>
-    <t>64,476.65</t>
-  </si>
-  <si>
     <t>บนบก</t>
   </si>
   <si>
@@ -388,28 +381,10 @@
     <t>รวมอัตราการผลิตบนบก</t>
   </si>
   <si>
-    <t>23,167.69</t>
-  </si>
-  <si>
-    <t>28,024.59</t>
-  </si>
-  <si>
     <t>รวมอัตราการผลิตทั้งหมด</t>
   </si>
   <si>
     <t>2,602.17</t>
-  </si>
-  <si>
-    <t>453,818.72</t>
-  </si>
-  <si>
-    <t>73,801.57</t>
-  </si>
-  <si>
-    <t>67,129.91</t>
-  </si>
-  <si>
-    <t>92,501.25</t>
   </si>
   <si>
     <t>613,449.87 บาร์เรล/วัน</t>
@@ -451,14 +426,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -469,37 +439,56 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -789,49 +778,74 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J43"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.283447" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="21.137695" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="39.990234" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="19.995117" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="23.422852" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="16.424561" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="23.422852" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="18.709717" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="18.709717" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="10.568848" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="2" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="D4" s="1" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="E4" s="4"/>
+      <c r="F4" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -863,7 +877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
@@ -893,7 +907,7 @@
       </c>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -923,7 +937,7 @@
       </c>
       <c r="J7" s="2"/>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -953,7 +967,7 @@
       </c>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -983,7 +997,7 @@
       </c>
       <c r="J9" s="2"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
@@ -1013,7 +1027,7 @@
       </c>
       <c r="J10" s="2"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>14</v>
       </c>
@@ -1024,7 +1038,7 @@
         <v>35</v>
       </c>
       <c r="D11" s="2">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E11" s="2">
         <v>25.15</v>
@@ -1043,7 +1057,7 @@
       </c>
       <c r="J11" s="2"/>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>14</v>
       </c>
@@ -1073,7 +1087,7 @@
       </c>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
@@ -1103,7 +1117,7 @@
       </c>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -1133,7 +1147,7 @@
       </c>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -1163,7 +1177,7 @@
       </c>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -1193,7 +1207,7 @@
       </c>
       <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>14</v>
       </c>
@@ -1223,7 +1237,7 @@
       </c>
       <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>14</v>
       </c>
@@ -1253,7 +1267,7 @@
       </c>
       <c r="J18" s="2"/>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>14</v>
       </c>
@@ -1283,7 +1297,7 @@
       </c>
       <c r="J19" s="2"/>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>14</v>
       </c>
@@ -1313,7 +1327,7 @@
       </c>
       <c r="J20" s="2"/>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>14</v>
       </c>
@@ -1343,7 +1357,7 @@
       </c>
       <c r="J21" s="2"/>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>14</v>
       </c>
@@ -1373,7 +1387,7 @@
       </c>
       <c r="J22" s="2"/>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>14</v>
       </c>
@@ -1403,7 +1417,7 @@
       </c>
       <c r="J23" s="2"/>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>14</v>
       </c>
@@ -1433,7 +1447,7 @@
       </c>
       <c r="J24" s="2"/>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>14</v>
       </c>
@@ -1463,7 +1477,7 @@
       </c>
       <c r="J25" s="2"/>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>14</v>
       </c>
@@ -1493,7 +1507,7 @@
       </c>
       <c r="J26" s="2"/>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>14</v>
       </c>
@@ -1523,37 +1537,39 @@
       </c>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:10">
-      <c r="A28" s="2" t="s">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
         <v>89</v>
       </c>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
       <c r="D28" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>94</v>
+      <c r="E28" s="7">
+        <v>430651.03</v>
+      </c>
+      <c r="F28" s="7">
+        <v>73584.55</v>
+      </c>
+      <c r="G28" s="7">
+        <v>66932.509999999995</v>
+      </c>
+      <c r="H28" s="7">
+        <v>64476.65</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D29" s="2">
         <v>5.45</v>
@@ -1575,21 +1591,21 @@
       </c>
       <c r="J29" s="2"/>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C30" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="D30" s="2">
         <v>106.28</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F30" s="2">
         <v>217.02</v>
@@ -1605,15 +1621,15 @@
       </c>
       <c r="J30" s="2"/>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D31" s="2">
         <v>0.03</v>
@@ -1635,15 +1651,15 @@
       </c>
       <c r="J31" s="2"/>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D32" s="2">
         <v>0.12</v>
@@ -1665,15 +1681,15 @@
       </c>
       <c r="J32" s="2"/>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D33" s="2">
         <v>0.21</v>
@@ -1688,22 +1704,22 @@
         <v>0</v>
       </c>
       <c r="H33" s="2">
-        <v>546.19</v>
+        <v>546.19000000000005</v>
       </c>
       <c r="I33" s="2">
         <v>31</v>
       </c>
       <c r="J33" s="2"/>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D34" s="2">
         <v>0.13</v>
@@ -1725,15 +1741,15 @@
       </c>
       <c r="J34" s="2"/>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D35" s="2">
         <v>0</v>
@@ -1755,21 +1771,21 @@
       </c>
       <c r="J35" s="2"/>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D36" s="2">
         <v>0.06</v>
       </c>
       <c r="E36" s="2">
-        <v>10.13</v>
+        <v>10.130000000000001</v>
       </c>
       <c r="F36" s="2">
         <v>0</v>
@@ -1778,22 +1794,22 @@
         <v>0</v>
       </c>
       <c r="H36" s="2">
-        <v>156.48</v>
+        <v>156.47999999999999</v>
       </c>
       <c r="I36" s="2">
         <v>31</v>
       </c>
       <c r="J36" s="2"/>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="D37" s="2">
         <v>0</v>
@@ -1815,15 +1831,15 @@
       </c>
       <c r="J37" s="2"/>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D38" s="2">
         <v>0.16</v>
@@ -1838,28 +1854,28 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="I38" s="2">
         <v>31</v>
       </c>
       <c r="J38" s="2"/>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D39" s="2">
         <v>20.41</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F39" s="2">
         <v>0</v>
@@ -1868,22 +1884,24 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I39" s="2">
         <v>31</v>
       </c>
       <c r="J39" s="2"/>
     </row>
-    <row r="40" spans="1:10">
-      <c r="A40" s="2" t="s">
-        <v>122</v>
-      </c>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
       <c r="D40" s="2">
         <v>132.84</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>123</v>
+      <c r="E40" s="7">
+        <v>23167.69</v>
       </c>
       <c r="F40" s="2">
         <v>217.02</v>
@@ -1891,72 +1909,80 @@
       <c r="G40" s="2">
         <v>197.4</v>
       </c>
-      <c r="H40" s="2" t="s">
-        <v>124</v>
+      <c r="H40" s="7">
+        <v>28024.59</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
     </row>
-    <row r="41" spans="1:10">
-      <c r="A41" s="2" t="s">
-        <v>125</v>
-      </c>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
       <c r="D41" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>130</v>
+        <v>120</v>
+      </c>
+      <c r="E41" s="7">
+        <v>453818.72</v>
+      </c>
+      <c r="F41" s="7">
+        <v>73801.570000000007</v>
+      </c>
+      <c r="G41" s="7">
+        <v>67129.91</v>
+      </c>
+      <c r="H41" s="7">
+        <v>92501.25</v>
       </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
     </row>
-    <row r="42" spans="1:10">
-      <c r="A42" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10">
-      <c r="A43" s="3" t="s">
-        <v>132</v>
-      </c>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="4"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
-  <mergeCells>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <mergeCells count="11">
+    <mergeCell ref="A43:J43"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="D42:I42"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A40:C40"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="D42:I42"/>
-    <mergeCell ref="A43:J43"/>
   </mergeCells>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>